<commit_message>
tiny wording rubric edit
</commit_message>
<xml_diff>
--- a/docs/2627/report/dapr3_2627_report_rubric.xlsx
+++ b/docs/2627/report/dapr3_2627_report_rubric.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jking34\Desktop\uoepsy_courses\dapr3\docs\2627\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F90261-3C3E-458E-9EAC-6C7725B7541A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE4927B-3A01-4B96-983B-F6EBCB22CCD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-25485" yWindow="-1110" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{80E36928-E358-2446-BA2E-DC98679EB28E}"/>
+    <workbookView xWindow="-28920" yWindow="-2805" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{80E36928-E358-2446-BA2E-DC98679EB28E}"/>
     <workbookView xWindow="-28920" yWindow="-2805" windowWidth="29040" windowHeight="15720" xr2:uid="{6478FE4C-0DDA-3A4B-B07C-63BB646B301E}"/>
   </bookViews>
   <sheets>
@@ -297,7 +297,7 @@
     <t>You introduce each figure and table in the text and cross-reference their numbers appropriately (including figures shown in the Appendix).</t>
   </si>
   <si>
-    <t>You accurately interpret the estimated quantity(ies) from your analysis to address the RQ(s)/hypothesis(es).</t>
+    <t>You accurately interpret the estimated quantity/quantities from your analysis to address each RQ/prediction.</t>
   </si>
 </sst>
 </file>
@@ -897,7 +897,7 @@
         <v>No entries!</v>
       </c>
       <c r="I2" s="4">
-        <f>IF($C2=1, 3, IF($D2=1, 2, IF($E2=1, 1, IF($F2 = 1, 0, 0))))</f>
+        <f t="shared" ref="I2:I21" si="1">IF($C2=1, 3, IF($D2=1, 2, IF($E2=1, 1, IF($F2 = 1, 0, 0))))</f>
         <v>0</v>
       </c>
     </row>
@@ -917,7 +917,7 @@
         <v>No entries!</v>
       </c>
       <c r="I3" s="4">
-        <f>IF($C3=1, 3, IF($D3=1, 2, IF($E3=1, 1, IF($F3 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -937,7 +937,7 @@
         <v>No entries!</v>
       </c>
       <c r="I4" s="4">
-        <f>IF($C4=1, 3, IF($D4=1, 2, IF($E4=1, 1, IF($F4 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -957,7 +957,7 @@
         <v>No entries!</v>
       </c>
       <c r="I5" s="4">
-        <f>IF($C5=1, 3, IF($D5=1, 2, IF($E5=1, 1, IF($F5 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -977,7 +977,7 @@
         <v>No entries!</v>
       </c>
       <c r="I6" s="4">
-        <f>IF($C6=1, 3, IF($D6=1, 2, IF($E6=1, 1, IF($F6 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M6" s="26"/>
@@ -1000,7 +1000,7 @@
         <v>No entries!</v>
       </c>
       <c r="I7" s="4">
-        <f>IF($C7=1, 3, IF($D7=1, 2, IF($E7=1, 1, IF($F7 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M7" s="26"/>
@@ -1023,7 +1023,7 @@
         <v>No entries!</v>
       </c>
       <c r="I8" s="4">
-        <f>IF($C8=1, 3, IF($D8=1, 2, IF($E8=1, 1, IF($F8 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M8" s="26"/>
@@ -1046,7 +1046,7 @@
         <v>No entries!</v>
       </c>
       <c r="I9" s="4">
-        <f>IF($C9=1, 3, IF($D9=1, 2, IF($E9=1, 1, IF($F9 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
         <v>No entries!</v>
       </c>
       <c r="I10" s="4">
-        <f>IF($C10=1, 3, IF($D10=1, 2, IF($E10=1, 1, IF($F10 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
         <v>No entries!</v>
       </c>
       <c r="I11" s="4">
-        <f>IF($C11=1, 3, IF($D11=1, 2, IF($E11=1, 1, IF($F11 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
         <v>No entries!</v>
       </c>
       <c r="I12" s="4">
-        <f>IF($C12=1, 3, IF($D12=1, 2, IF($E12=1, 1, IF($F12 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
         <v>No entries!</v>
       </c>
       <c r="I13" s="4">
-        <f>IF($C13=1, 3, IF($D13=1, 2, IF($E13=1, 1, IF($F13 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         <v>No entries!</v>
       </c>
       <c r="I14" s="4">
-        <f>IF($C14=1, 3, IF($D14=1, 2, IF($E14=1, 1, IF($F14 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1166,7 +1166,7 @@
         <v>No entries!</v>
       </c>
       <c r="I15" s="4">
-        <f>IF($C15=1, 3, IF($D15=1, 2, IF($E15=1, 1, IF($F15 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
         <v>No entries!</v>
       </c>
       <c r="I16" s="4">
-        <f>IF($C16=1, 3, IF($D16=1, 2, IF($E16=1, 1, IF($F16 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
         <v>No entries!</v>
       </c>
       <c r="I17" s="4">
-        <f>IF($C17=1, 3, IF($D17=1, 2, IF($E17=1, 1, IF($F17 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>No entries!</v>
       </c>
       <c r="I18" s="4">
-        <f>IF($C18=1, 3, IF($D18=1, 2, IF($E18=1, 1, IF($F18 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
         <v>No entries!</v>
       </c>
       <c r="I19" s="4">
-        <f>IF($C19=1, 3, IF($D19=1, 2, IF($E19=1, 1, IF($F19 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
         <v>No entries!</v>
       </c>
       <c r="I20" s="4">
-        <f>IF($C20=1, 3, IF($D20=1, 2, IF($E20=1, 1, IF($F20 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
         <v>No entries!</v>
       </c>
       <c r="I21" s="4">
-        <f>IF($C21=1, 3, IF($D21=1, 2, IF($E21=1, 1, IF($F21 = 1, 0, 0))))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>